<commit_message>
further parameter calibration plus sensitivity tests added
</commit_message>
<xml_diff>
--- a/Prototypes/Sesame/SesameObserved.xlsx
+++ b/Prototypes/Sesame/SesameObserved.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\source\repos\Sesame-Apsimx\Apsimx\Prototypes\Sesame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A2AEFF0-7539-44DD-B876-E99674964D26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41CE37C9-E702-48D7-B23D-1AA5832E51BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="700" yWindow="1120" windowWidth="24390" windowHeight="14150" xr2:uid="{857C0208-4D04-4514-A3CE-6D305A175862}"/>
+    <workbookView xWindow="39465" yWindow="120" windowWidth="24870" windowHeight="15585" xr2:uid="{857C0208-4D04-4514-A3CE-6D305A175862}"/>
   </bookViews>
   <sheets>
     <sheet name="Observed" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="88">
   <si>
     <t>SimulationName</t>
   </si>
@@ -275,6 +275,30 @@
   </si>
   <si>
     <t>PopRelativeError%</t>
+  </si>
+  <si>
+    <t>EmeraldGNS25_S57B</t>
+  </si>
+  <si>
+    <t>EmeraldGNS25_ES103</t>
+  </si>
+  <si>
+    <t>EmeraldGNS25_S3301</t>
+  </si>
+  <si>
+    <t>EmeraldGNS25_S3313</t>
+  </si>
+  <si>
+    <t>EmeraldGNS25N_0</t>
+  </si>
+  <si>
+    <t>EmeraldGNS25N_40</t>
+  </si>
+  <si>
+    <t>EmeraldGNS25N_80</t>
+  </si>
+  <si>
+    <t>EmeraldGNS25N_120</t>
   </si>
 </sst>
 </file>
@@ -349,7 +373,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -401,6 +425,15 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -716,7 +749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E72B3C1-BBAB-449C-BAE0-DBB067DF5460}">
-  <dimension ref="A1:U146"/>
+  <dimension ref="A1:U154"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.81640625" style="2" bestFit="1" customWidth="1"/>
@@ -1201,7 +1234,9 @@
       <c r="A19" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="12"/>
+      <c r="B19" s="12">
+        <v>45033</v>
+      </c>
       <c r="C19" s="5" t="s">
         <v>6</v>
       </c>
@@ -1230,7 +1265,9 @@
       <c r="A20" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="12"/>
+      <c r="B20" s="12">
+        <v>45153</v>
+      </c>
       <c r="C20" s="5" t="s">
         <v>3</v>
       </c>
@@ -1259,7 +1296,9 @@
       <c r="A21" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="12"/>
+      <c r="B21" s="12">
+        <v>45178</v>
+      </c>
       <c r="C21" s="5" t="s">
         <v>19</v>
       </c>
@@ -1315,6 +1354,9 @@
       <c r="A22" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="B22" s="8">
+        <v>45026</v>
+      </c>
       <c r="C22" s="2" t="s">
         <v>6</v>
       </c>
@@ -1326,6 +1368,9 @@
       <c r="A23" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="B23" s="8">
+        <v>45148</v>
+      </c>
       <c r="C23" s="2" t="s">
         <v>3</v>
       </c>
@@ -1337,6 +1382,9 @@
       <c r="A24" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="B24" s="8">
+        <v>45188</v>
+      </c>
       <c r="C24" s="2" t="s">
         <v>19</v>
       </c>
@@ -1498,6 +1546,9 @@
     <row r="27" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>23</v>
+      </c>
+      <c r="B27" s="8">
+        <v>46162</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>12</v>
@@ -4602,6 +4653,154 @@
       <c r="S146" s="11"/>
       <c r="T146" s="11"/>
       <c r="U146" s="11"/>
+    </row>
+    <row r="147" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A147" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B147" s="8">
+        <v>46050</v>
+      </c>
+      <c r="D147" s="2">
+        <v>99</v>
+      </c>
+      <c r="H147" s="2">
+        <v>363</v>
+      </c>
+      <c r="L147" s="2">
+        <v>48.1</v>
+      </c>
+    </row>
+    <row r="148" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A148" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B148" s="8">
+        <v>46050</v>
+      </c>
+      <c r="D148" s="2">
+        <v>99</v>
+      </c>
+      <c r="H148" s="2">
+        <v>526</v>
+      </c>
+      <c r="L148" s="2">
+        <v>92.5</v>
+      </c>
+    </row>
+    <row r="149" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A149" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B149" s="8">
+        <v>46050</v>
+      </c>
+      <c r="D149" s="2">
+        <v>99</v>
+      </c>
+      <c r="H149" s="2">
+        <v>472</v>
+      </c>
+      <c r="L149" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="150" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A150" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B150" s="8">
+        <v>46050</v>
+      </c>
+      <c r="D150" s="2">
+        <v>99</v>
+      </c>
+      <c r="H150" s="2">
+        <v>336</v>
+      </c>
+      <c r="L150" s="2">
+        <v>61.9</v>
+      </c>
+    </row>
+    <row r="151" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A151" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B151" s="8">
+        <v>46050</v>
+      </c>
+      <c r="D151" s="2">
+        <v>99</v>
+      </c>
+      <c r="H151" s="20">
+        <v>290.5</v>
+      </c>
+      <c r="I151" s="18"/>
+      <c r="J151" s="18"/>
+      <c r="K151" s="19"/>
+      <c r="L151" s="20">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="152" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A152" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B152" s="8">
+        <v>46050</v>
+      </c>
+      <c r="D152" s="2">
+        <v>99</v>
+      </c>
+      <c r="H152" s="20">
+        <v>390</v>
+      </c>
+      <c r="I152" s="18"/>
+      <c r="J152" s="18"/>
+      <c r="K152" s="19"/>
+      <c r="L152" s="20">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="153" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A153" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B153" s="8">
+        <v>46050</v>
+      </c>
+      <c r="D153" s="2">
+        <v>99</v>
+      </c>
+      <c r="H153" s="20">
+        <v>325.5</v>
+      </c>
+      <c r="I153" s="18"/>
+      <c r="J153" s="18"/>
+      <c r="K153" s="19"/>
+      <c r="L153" s="20">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="154" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A154" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B154" s="8">
+        <v>46050</v>
+      </c>
+      <c r="D154" s="2">
+        <v>99</v>
+      </c>
+      <c r="H154" s="20">
+        <v>351</v>
+      </c>
+      <c r="I154" s="18"/>
+      <c r="J154" s="18"/>
+      <c r="K154" s="19"/>
+      <c r="L154" s="20">
+        <v>62.5</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U235">

</xml_diff>